<commit_message>
docs(school): add Sprint & PB (backlog) IDs to WS5 test artifacts
Make the four IDs cross-reference the real backlog: test case ID, PB
(product backlog task), Sprint ID, and RQ (user story) now match the
"ws4.1 sprints" sheet of 2607lts nhóm 1 WebBshoes.xlsx exactly.

- TestCase.xlsx: each module sheet header shows Sprint + PB; Test Case
  List becomes a Sprint -> PB -> RQ -> Test case traceability matrix.
- DefectReport.xlsx: group headers show module PB / Sprint / RQ.
- WORKSHOP_5_BShoes.docx: scope and traceability tables gain Sprint + PB
  columns.

Mapping: DN=pb-1/S1, NV=pb-2/S1, SP+DMTT=pb-3/S1, KHO=PB-4/S1,
POS+GH=PB-5/S2, PGG=PB-6/S2, TH=PB-7/S3, KH=PB-8/S3.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc-school/ws5/BShoes_DefectReport.xlsx
+++ b/doc-school/ws5/BShoes_DefectReport.xlsx
@@ -129,7 +129,7 @@
     <t>Related Testcase ID</t>
   </si>
   <si>
-    <t>Module: Đăng nhập (Sprint 3 - TEST)</t>
+    <t>Module: Đăng nhập — pb-1 / Sprint 1 / RQ-1  (phát hiện ở Sprint 3 - TEST)</t>
   </si>
   <si>
     <t>BUG_DN_01</t>
@@ -164,7 +164,7 @@
     <t>DN_13</t>
   </si>
   <si>
-    <t>Module: Quản lý nhân viên (Sprint 3 - TEST)</t>
+    <t>Module: Quản lý nhân viên — pb-2 / Sprint 1 / RQ-2,RQ-3,RQ-4  (phát hiện ở Sprint 3 - TEST)</t>
   </si>
   <si>
     <t>BUG_NV_01</t>
@@ -196,7 +196,7 @@
     <t>NV_08</t>
   </si>
   <si>
-    <t>Module: Quản lý sản phẩm (Sprint 3 - TEST)</t>
+    <t>Module: Quản lý sản phẩm — pb-3 / Sprint 1 / RQ-5,RQ-6,RQ-9  (phát hiện ở Sprint 3 - TEST)</t>
   </si>
   <si>
     <t>BUG_SP_01</t>
@@ -239,7 +239,7 @@
     <t>SP_13</t>
   </si>
   <si>
-    <t>Module: Bán hàng - POS (Sprint 3 - TEST)</t>
+    <t>Module: Bán hàng POS — PB-5 / Sprint 2 / RQ-11→RQ-18  (phát hiện ở Sprint 3 - TEST)</t>
   </si>
   <si>
     <t>BUG_POS_01</t>
@@ -284,7 +284,7 @@
     <t>POS_19</t>
   </si>
   <si>
-    <t>Module: Quản lý phiếu giảm giá (Sprint 3 - TEST)</t>
+    <t>Module: Quản lý phiếu giảm giá — PB-6 / Sprint 2 / RQ-21  (phát hiện ở Sprint 3 - TEST)</t>
   </si>
   <si>
     <t>BUG_PGG_01</t>
@@ -304,7 +304,7 @@
     <t>PGG_05</t>
   </si>
   <si>
-    <t>Module: Quản lý trả hàng (Sprint 3 - TEST)</t>
+    <t>Module: Quản lý trả hàng — PB-7 / Sprint 3 / RQ-22  (phát hiện ở Sprint 3 - TEST)</t>
   </si>
   <si>
     <t>BUG_TH_01</t>

</xml_diff>